<commit_message>
feat(enterprise): import Excel (.xlsx) de la flotte depuis le tableau de bord
Étend l'import véhicules existant pour accepter le modèle d'onboarding
.xlsx en plus du CSV : lecture de la feuille « Véhicules » via exceljs,
normalisation des en-têtes (« Marque * », « Type d'usage », « Groupe /
Site »), logique de validation partagée entre CSV et XLSX. La route
détecte le format par extension/mimetype.

Le modèle est régénéré sans ligne d'indices (indices passés en
commentaires de cellule, données dès la ligne 2) pour être importable
proprement, et servi en téléchargement depuis la page d'import.

Codes d'erreur CSV_* renommés IMPORT_* (communs aux deux formats).
3 nouveaux tests XLSX ; 91 tests enterprise verts.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/onboarding/modele-onboarding-flotte.xlsx
+++ b/docs/onboarding/modele-onboarding-flotte.xlsx
@@ -107,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,9 +123,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -201,6 +198,101 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Pièces</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Toyota, Hyundai…</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Hilux, H1…</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>2018</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>1234 AB 01</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>N° de châssis (17 car.)</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>2.5 D-4D, essence…</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>en km</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>voir liste</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>ex : Dépôt Nord</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>nom du chauffeur</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Pièces</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Prénom Nom</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>+2250700000000</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>B, C, D…</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>JJ/MM/AAAA</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>remarques</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -846,56 +938,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>Toyota, Hyundai…</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>Hilux, H1…</t>
-        </is>
-      </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="inlineStr">
-        <is>
-          <t>1234 AB 01</t>
-        </is>
-      </c>
-      <c r="E2" s="10" t="inlineStr">
-        <is>
-          <t>N° de châssis (17 car.)</t>
-        </is>
-      </c>
-      <c r="F2" s="10" t="inlineStr">
-        <is>
-          <t>2.5 D-4D, essence…</t>
-        </is>
-      </c>
-      <c r="G2" s="10" t="inlineStr">
-        <is>
-          <t>en km</t>
-        </is>
-      </c>
-      <c r="H2" s="10" t="inlineStr">
-        <is>
-          <t>voir liste</t>
-        </is>
-      </c>
-      <c r="I2" s="10" t="inlineStr">
-        <is>
-          <t>ex : Dépôt Nord</t>
-        </is>
-      </c>
-      <c r="J2" s="10" t="inlineStr">
-        <is>
-          <t>nom du chauffeur</t>
-        </is>
-      </c>
+      <c r="A2" s="7" t="n"/>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
+      <c r="J2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n"/>
@@ -1583,15 +1635,16 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="H3:H59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRANSPORT,CHANTIER,LIVRAISON,DIRECTION,AUTRE"</formula1>
     </dataValidation>
-    <dataValidation sqref="C3:C59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="C2:C59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1980</formula1>
       <formula2>2030</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1645,31 +1698,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>Prénom Nom</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>+2250700000000</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="inlineStr">
-        <is>
-          <t>B, C, D…</t>
-        </is>
-      </c>
-      <c r="E2" s="10" t="inlineStr">
-        <is>
-          <t>JJ/MM/AAAA</t>
-        </is>
-      </c>
-      <c r="F2" s="10" t="inlineStr">
-        <is>
-          <t>remarques</t>
-        </is>
-      </c>
+      <c r="A2" s="7" t="n"/>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n"/>
@@ -1969,5 +2003,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>